<commit_message>
Improve CDB bid parsing and recover additional contract USD amounts
</commit_message>
<xml_diff>
--- a/data/raw/cdb/cdb_lac_raw.xlsx
+++ b/data/raw/cdb/cdb_lac_raw.xlsx
@@ -1051,13 +1051,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Drip Irrigation XCD 1,755,</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
+          <t>Drip Irrigation</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>XCD</t>
+        </is>
+      </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>802.75</t>
+          <t>1755802.75</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -2122,13 +2126,17 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>M&amp;amp;R Construction L imited BZD 1,</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr"/>
+          <t>M&amp;amp;R Construction L imited</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>298576.42</t>
+          <t>1298576.42</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
@@ -2187,13 +2195,17 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Teichroeb &amp;amp; Sons Limited BZD 2,</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr"/>
+          <t>Teichroeb &amp;amp; Sons Limited</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>539571.76</t>
+          <t>2539571.76</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
@@ -2954,16 +2966,24 @@
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Caribbean DMS, in association with Community Systems Foundation USD 73,</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr"/>
+          <t>Caribbean DMS, in association with Community Systems Foundation</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>280.0</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr"/>
+          <t>73280.0</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>73280.0</t>
+        </is>
+      </c>
       <c r="M36" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/Contract-Award-Information_DevInfo-Training-Workshops1.pdf</t>
@@ -4767,13 +4787,17 @@
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Surrey Paving and Aggregate Co. Ltd. JA$ 1,176,184,636 .</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr"/>
+          <t>Surrey Paving and Aggregate Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>JA$</t>
+        </is>
+      </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>1176184636.05</t>
         </is>
       </c>
       <c r="L61" t="inlineStr"/>
@@ -5213,16 +5237,24 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>- Sumec, Complete Equipment &amp;amp; Engineering Co.,Ltd. US$8,</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr"/>
+          <t>- Sumec, Complete Equipment &amp;amp; Engineering Co.,Ltd.</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>US$</t>
+        </is>
+      </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>306324.0</t>
-        </is>
-      </c>
-      <c r="L67" t="inlineStr"/>
+          <t>8306324.0</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>8306324.0</t>
+        </is>
+      </c>
       <c r="M67" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/CONTRACT_AWARD_INFORMATION%20_SOLAR%20PLANTS_V2.pdf</t>
@@ -6644,7 +6676,7 @@
       <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr">
         <is>
-          <t>USD 4,527,140.00</t>
+          <t>USD 22,000</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -6654,12 +6686,12 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>22000.0</t>
+          <t>4527140.0</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>22000.0</t>
+          <t>4527140.0</t>
         </is>
       </c>
       <c r="M86" t="inlineStr"/>
@@ -7963,12 +7995,12 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>-Island Site Development Ltd</t>
+          <t>-Island Site Development Ltd BAH</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>BAH</t>
+          <t>$</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -9025,13 +9057,17 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>- BAE CONSTRUCTION BZD$ 1, 134,</t>
-        </is>
-      </c>
-      <c r="J119" t="inlineStr"/>
+          <t>- BAE CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
       <c r="K119" t="inlineStr">
         <is>
-          <t>920.0</t>
+          <t>1134920.0</t>
         </is>
       </c>
       <c r="L119" t="inlineStr"/>
@@ -9467,12 +9503,12 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Champion Security Systems Li</t>
+          <t>Champion Security Systems Limited</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>mited</t>
+          <t>$</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -9480,7 +9516,11 @@
           <t>28802.25</t>
         </is>
       </c>
-      <c r="L125" t="inlineStr"/>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>28802.25</t>
+        </is>
+      </c>
       <c r="M125" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/Contract-Award-Information%20-%20Security%20Cameras.pdf</t>
@@ -9901,13 +9941,17 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>- Franco Construction Ltd XCD 1,</t>
-        </is>
-      </c>
-      <c r="J131" t="inlineStr"/>
+          <t>- Franco Construction Ltd</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>XCD</t>
+        </is>
+      </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>484645.83</t>
+          <t>1484645.83</t>
         </is>
       </c>
       <c r="L131" t="inlineStr"/>
@@ -10274,12 +10318,12 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Diesel and Equipment Company Limited</t>
+          <t>Diesel and Equipment Company Limited BDZ</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>BDZ</t>
+          <t>$</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -10289,7 +10333,7 @@
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>1113887.25</t>
+          <t>2227774.5</t>
         </is>
       </c>
       <c r="M136" t="inlineStr">
@@ -10351,7 +10395,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>- Massy Technologies for Lot 1, and BVI- Island Services BVI Limited for Lot 3 a &amp;amp; b. Lot 1: $257,450.00 Lot 3 a &amp;amp; b:</t>
+          <t>- Massy Technologies for Lot 1, and BVI- Island Services BVI Limited for Lot 3 a &amp;amp; b. Lot 1: Lot 3 a &amp;amp; b: $618,325.12</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -10361,12 +10405,12 @@
       </c>
       <c r="K137" t="inlineStr">
         <is>
-          <t>618325.12</t>
+          <t>257450.0</t>
         </is>
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>618325.12</t>
+          <t>257450.0</t>
         </is>
       </c>
       <c r="M137" t="inlineStr">
@@ -11117,12 +11161,24 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>- Integrated Sustainability USD119,920.00 plus applicable VAT and Foreign Exchange Levy</t>
-        </is>
-      </c>
-      <c r="J147" t="inlineStr"/>
-      <c r="K147" t="inlineStr"/>
-      <c r="L147" t="inlineStr"/>
+          <t>- Integrated Sustainability plus applicable VAT and Foreign Exchange Levy</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>119920.0</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>119920.0</t>
+        </is>
+      </c>
       <c r="M147" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/BAR_GAIA%20Pavement%20Rehab_CS_Sustainability%20Mgmt%20Plan_CAI_AMH%2004102021.pdf</t>
@@ -12747,11 +12803,19 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>- Stewart Engineering Limited XCD 393,610.00 (Tax Exclusive)</t>
-        </is>
-      </c>
-      <c r="J169" t="inlineStr"/>
-      <c r="K169" t="inlineStr"/>
+          <t>- Stewart Engineering Limited (Tax Exclusive)</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>XCD</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>393610.0</t>
+        </is>
+      </c>
       <c r="L169" t="inlineStr"/>
       <c r="M169" t="inlineStr">
         <is>
@@ -12889,11 +12953,19 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>- Gleans Construction and Engineering Co. Limited XCD 460,000.00 (Tax Exclusive)</t>
-        </is>
-      </c>
-      <c r="J171" t="inlineStr"/>
-      <c r="K171" t="inlineStr"/>
+          <t>- Gleans Construction and Engineering Co. Limited (Tax Exclusive)</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>XCD</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>460000.0</t>
+        </is>
+      </c>
       <c r="L171" t="inlineStr"/>
       <c r="M171" t="inlineStr">
         <is>
@@ -12954,11 +13026,19 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>- Gleans Construction and Engineering Co. Limited XCD 290,000.00 (Tax Exclusive)</t>
-        </is>
-      </c>
-      <c r="J172" t="inlineStr"/>
-      <c r="K172" t="inlineStr"/>
+          <t>- Gleans Construction and Engineering Co. Limited (Tax Exclusive)</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>XCD</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>290000.0</t>
+        </is>
+      </c>
       <c r="L172" t="inlineStr"/>
       <c r="M172" t="inlineStr">
         <is>
@@ -13315,16 +13395,24 @@
       <c r="H177" t="inlineStr"/>
       <c r="I177" t="inlineStr">
         <is>
-          <t>HR Wallingford Ltd. USD 30,</t>
-        </is>
-      </c>
-      <c r="J177" t="inlineStr"/>
+          <t>HR Wallingford Ltd.</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="L177" t="inlineStr"/>
+          <t>30000.0</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>30000.0</t>
+        </is>
+      </c>
       <c r="M177" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/Award%20of%20Contract_HR%20Wallingford%20Consultants.pdf</t>
@@ -19408,11 +19496,19 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>- Anthony Thurton and Associates Ltd. BZD 251,887.50 (Inclusive of taxes)</t>
-        </is>
-      </c>
-      <c r="J262" t="inlineStr"/>
-      <c r="K262" t="inlineStr"/>
+          <t>- Anthony Thurton and Associates Ltd. (Inclusive of taxes)</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>251887.5</t>
+        </is>
+      </c>
       <c r="L262" t="inlineStr"/>
       <c r="M262" t="inlineStr">
         <is>
@@ -19903,16 +19999,24 @@
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>- Aecon Construction Group Inc. USD155, 303, 809. 73 &amp;amp; EUR12, 306,</t>
-        </is>
-      </c>
-      <c r="J269" t="inlineStr"/>
+          <t>- Aecon Construction Group Inc. &amp;amp; EUR12,306,636.14</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
       <c r="K269" t="inlineStr">
         <is>
-          <t>636.14</t>
-        </is>
-      </c>
-      <c r="L269" t="inlineStr"/>
+          <t>155303809.73</t>
+        </is>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>155303809.73</t>
+        </is>
+      </c>
       <c r="M269" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/220405_SVG_Kingstown%20Port%20Modernisation%20Project_W_Design%20%20Build%20Contractor_1.pdf</t>
@@ -19972,13 +20076,17 @@
       </c>
       <c r="I270" t="inlineStr">
         <is>
-          <t>- Sellhorn Ingenieurgesellschaft mbH EUR3, 884,</t>
-        </is>
-      </c>
-      <c r="J270" t="inlineStr"/>
+          <t>- Sellhorn Ingenieurgesellschaft mbH</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
       <c r="K270" t="inlineStr">
         <is>
-          <t>905.0</t>
+          <t>3884905.0</t>
         </is>
       </c>
       <c r="L270" t="inlineStr"/>
@@ -21460,12 +21568,24 @@
       <c r="H290" t="inlineStr"/>
       <c r="I290" t="inlineStr">
         <is>
-          <t>Trinidad &amp;amp; Tobago - Odyssey Consultinc Limited USD $ 15,210.00 (exclusive of taxes)</t>
-        </is>
-      </c>
-      <c r="J290" t="inlineStr"/>
-      <c r="K290" t="inlineStr"/>
-      <c r="L290" t="inlineStr"/>
+          <t>Trinidad &amp;amp; Tobago - Odyssey Consultinc Limited (exclusive of taxes)</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>15210.0</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>15210.0</t>
+        </is>
+      </c>
       <c r="M290" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/Contract%20Award%20Information%281%29%20090823%20final.pdf</t>
@@ -21521,11 +21641,19 @@
       </c>
       <c r="I291" t="inlineStr">
         <is>
-          <t>- FDL Consult Inc. EC$630,085.00 (vat inclusive)</t>
-        </is>
-      </c>
-      <c r="J291" t="inlineStr"/>
-      <c r="K291" t="inlineStr"/>
+          <t>- FDL Consult Inc. (vat inclusive)</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>EC$</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>630085.0</t>
+        </is>
+      </c>
       <c r="L291" t="inlineStr"/>
       <c r="M291" t="inlineStr">
         <is>
@@ -21740,11 +21868,19 @@
       </c>
       <c r="I294" t="inlineStr">
         <is>
-          <t>- Bally and Bally Investment Ltd XCD $538,756.00 (Inclusive of taxes)</t>
-        </is>
-      </c>
-      <c r="J294" t="inlineStr"/>
-      <c r="K294" t="inlineStr"/>
+          <t>- Bally and Bally Investment Ltd (Inclusive of taxes)</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>XCD</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>538756.0</t>
+        </is>
+      </c>
       <c r="L294" t="inlineStr"/>
       <c r="M294" t="inlineStr">
         <is>
@@ -21805,12 +21941,24 @@
       </c>
       <c r="I295" t="inlineStr">
         <is>
-          <t>- Aecon Construction Group Inc US$ 155, 303, 809. 73 &amp;amp; EUR 12, 306, 663.14 (Exclusive of taxes)</t>
-        </is>
-      </c>
-      <c r="J295" t="inlineStr"/>
-      <c r="K295" t="inlineStr"/>
-      <c r="L295" t="inlineStr"/>
+          <t>- Aecon Construction Group Inc &amp;amp; EUR 12,306,663.14 (Exclusive of taxes)</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>US$</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>155303809.73</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>155303809.73</t>
+        </is>
+      </c>
       <c r="M295" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230525_SVG_CAI%20-Kingstown%20Port%20Modernisation%20Project%20-%20Design%20Build%20Contractor_Aecon%20.pdf</t>
@@ -21870,11 +22018,19 @@
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t>- Mitchell Moody Associates BZD $136,953.00 (Inclusive of taxes)</t>
-        </is>
-      </c>
-      <c r="J296" t="inlineStr"/>
-      <c r="K296" t="inlineStr"/>
+          <t>- Mitchell Moody Associates (Inclusive of taxes)</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>136953.0</t>
+        </is>
+      </c>
       <c r="L296" t="inlineStr"/>
       <c r="M296" t="inlineStr"/>
       <c r="N296" t="inlineStr">
@@ -22008,11 +22164,19 @@
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>- OB Sadoo Engineering Services Ltd. XCD 3,008,779.92 (Excluding VAT of XCD 376,097.49)</t>
-        </is>
-      </c>
-      <c r="J298" t="inlineStr"/>
-      <c r="K298" t="inlineStr"/>
+          <t>- OB Sadoo Engineering Services Ltd. (Excluding VAT of XCD 376,097.49)</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>XCD</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>3008779.92</t>
+        </is>
+      </c>
       <c r="L298" t="inlineStr"/>
       <c r="M298" t="inlineStr">
         <is>
@@ -22142,11 +22306,19 @@
       </c>
       <c r="I300" t="inlineStr">
         <is>
-          <t>- Anthony Thurton and Associates Ltd. BZD 242,720.33 (Inclusive of taxes)</t>
-        </is>
-      </c>
-      <c r="J300" t="inlineStr"/>
-      <c r="K300" t="inlineStr"/>
+          <t>- Anthony Thurton and Associates Ltd. (Inclusive of taxes)</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>242720.33</t>
+        </is>
+      </c>
       <c r="L300" t="inlineStr"/>
       <c r="M300" t="inlineStr">
         <is>
@@ -22203,11 +22375,19 @@
       </c>
       <c r="I301" t="inlineStr">
         <is>
-          <t>- Anthony Thurton and Associates Ltd. BZD 370,644.42 (Inclusive of taxes)</t>
-        </is>
-      </c>
-      <c r="J301" t="inlineStr"/>
-      <c r="K301" t="inlineStr"/>
+          <t>- Anthony Thurton and Associates Ltd. (Inclusive of taxes)</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>370644.42</t>
+        </is>
+      </c>
       <c r="L301" t="inlineStr"/>
       <c r="M301" t="inlineStr">
         <is>
@@ -22933,11 +23113,19 @@
       <c r="H311" t="inlineStr"/>
       <c r="I311" t="inlineStr">
         <is>
-          <t>St. Vincent &amp;amp; the Grenadines - Franco Construction Ltd XCD 6,060,539.03 (Revised Contract Amount)</t>
-        </is>
-      </c>
-      <c r="J311" t="inlineStr"/>
-      <c r="K311" t="inlineStr"/>
+          <t>St. Vincent &amp;amp; the Grenadines - Franco Construction Ltd (Revised Contract Amount)</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>XCD</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>6060539.03</t>
+        </is>
+      </c>
       <c r="L311" t="inlineStr"/>
       <c r="M311" t="inlineStr">
         <is>
@@ -22994,11 +23182,19 @@
       <c r="H312" t="inlineStr"/>
       <c r="I312" t="inlineStr">
         <is>
-          <t>St. Vincent &amp;amp; the Grenadines - Joint Venture (JV): Franco Construction Ltd and Sea Operations Ltd. XCD 3,539,883.14 (Revised Contract Amount)</t>
-        </is>
-      </c>
-      <c r="J312" t="inlineStr"/>
-      <c r="K312" t="inlineStr"/>
+          <t>St. Vincent &amp;amp; the Grenadines - Joint Venture (JV): Franco Construction Ltd and Sea Operations Ltd. (Revised Contract Amount)</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>XCD</t>
+        </is>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>3539883.14</t>
+        </is>
+      </c>
       <c r="L312" t="inlineStr"/>
       <c r="M312" t="inlineStr">
         <is>
@@ -23055,11 +23251,19 @@
       <c r="H313" t="inlineStr"/>
       <c r="I313" t="inlineStr">
         <is>
-          <t>St. Vincent &amp;amp; the Grenadines - Franco Construction Ltd XCD 2,069,326,.45 (Revised Contract Amount)</t>
-        </is>
-      </c>
-      <c r="J313" t="inlineStr"/>
-      <c r="K313" t="inlineStr"/>
+          <t>St. Vincent &amp;amp; the Grenadines - Franco Construction Ltd ,.45 (Revised Contract Amount)</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>XCD</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>2069326.0</t>
+        </is>
+      </c>
       <c r="L313" t="inlineStr"/>
       <c r="M313" t="inlineStr">
         <is>
@@ -23565,7 +23769,7 @@
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>Belize; Belize</t>
+          <t>Belize</t>
         </is>
       </c>
       <c r="I320" t="inlineStr">
@@ -24081,11 +24285,19 @@
       </c>
       <c r="I327" t="inlineStr">
         <is>
-          <t>- Young’s Engineering Consultancy Ltd BZD 351,123.76 (Inclusive of taxes)</t>
-        </is>
-      </c>
-      <c r="J327" t="inlineStr"/>
-      <c r="K327" t="inlineStr"/>
+          <t>- Young’s Engineering Consultancy Ltd (Inclusive of taxes)</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>351123.76</t>
+        </is>
+      </c>
       <c r="L327" t="inlineStr"/>
       <c r="M327" t="inlineStr">
         <is>
@@ -24287,16 +24499,24 @@
       </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t>Belize; Belize</t>
+          <t>Belize</t>
         </is>
       </c>
       <c r="I330" t="inlineStr">
         <is>
-          <t>Red Cross BZD $30,000.00 (inclusive of all taxes)</t>
-        </is>
-      </c>
-      <c r="J330" t="inlineStr"/>
-      <c r="K330" t="inlineStr"/>
+          <t>Red Cross (inclusive of all taxes)</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t>30000.0</t>
+        </is>
+      </c>
       <c r="L330" t="inlineStr"/>
       <c r="M330" t="inlineStr">
         <is>
@@ -24576,11 +24796,19 @@
       </c>
       <c r="I334" t="inlineStr">
         <is>
-          <t>- FDL Consult Inc XCD 454, 800.00 (Tax exclusive)</t>
-        </is>
-      </c>
-      <c r="J334" t="inlineStr"/>
-      <c r="K334" t="inlineStr"/>
+          <t>- FDL Consult Inc (Tax exclusive)</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>XCD</t>
+        </is>
+      </c>
+      <c r="K334" t="inlineStr">
+        <is>
+          <t>454800.0</t>
+        </is>
+      </c>
       <c r="L334" t="inlineStr"/>
       <c r="M334" t="inlineStr">
         <is>
@@ -24710,13 +24938,17 @@
       <c r="H336" t="inlineStr"/>
       <c r="I336" t="inlineStr">
         <is>
-          <t>USA - Pan American Health Organization (PAHO) BZD 368,334.</t>
-        </is>
-      </c>
-      <c r="J336" t="inlineStr"/>
+          <t>USA - Pan American Health Organization (PAHO) .00</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
       <c r="K336" t="inlineStr">
         <is>
-          <t>80.0</t>
+          <t>368334.8</t>
         </is>
       </c>
       <c r="L336" t="inlineStr"/>
@@ -24775,13 +25007,17 @@
       </c>
       <c r="I337" t="inlineStr">
         <is>
-          <t>- GS-COM BZD $29,</t>
-        </is>
-      </c>
-      <c r="J337" t="inlineStr"/>
+          <t>- GS-COM</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
       <c r="K337" t="inlineStr">
         <is>
-          <t>555.99</t>
+          <t>29555.99</t>
         </is>
       </c>
       <c r="L337" t="inlineStr"/>
@@ -24921,7 +25157,7 @@
       </c>
       <c r="I339" t="inlineStr">
         <is>
-          <t>- M and M Jamaica Ltd.</t>
+          <t>- M and M Jamaica Ltd. US</t>
         </is>
       </c>
       <c r="J339" t="inlineStr">
@@ -24998,12 +25234,12 @@
       </c>
       <c r="I340" t="inlineStr">
         <is>
-          <t>- Build Rite Construction Ltd.</t>
+          <t>- Build Rite Construction Ltd. US</t>
         </is>
       </c>
       <c r="J340" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>$</t>
         </is>
       </c>
       <c r="K340" t="inlineStr">
@@ -25379,11 +25615,19 @@
       </c>
       <c r="I345" t="inlineStr">
         <is>
-          <t>- Young’s Engineering Consultancy Ltd. BZD $154,849.50 (inclusive of all taxes)</t>
-        </is>
-      </c>
-      <c r="J345" t="inlineStr"/>
-      <c r="K345" t="inlineStr"/>
+          <t>- Young’s Engineering Consultancy Ltd. (inclusive of all taxes)</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
+      <c r="K345" t="inlineStr">
+        <is>
+          <t>154849.5</t>
+        </is>
+      </c>
       <c r="L345" t="inlineStr"/>
       <c r="M345" t="inlineStr">
         <is>
@@ -25440,11 +25684,19 @@
       </c>
       <c r="I346" t="inlineStr">
         <is>
-          <t>- Anthony Thurton and Associates Ltd. BZD $189,787.50 (inclusive of all taxes)</t>
-        </is>
-      </c>
-      <c r="J346" t="inlineStr"/>
-      <c r="K346" t="inlineStr"/>
+          <t>- Anthony Thurton and Associates Ltd. (inclusive of all taxes)</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
+      <c r="K346" t="inlineStr">
+        <is>
+          <t>189787.5</t>
+        </is>
+      </c>
       <c r="L346" t="inlineStr"/>
       <c r="M346" t="inlineStr">
         <is>
@@ -25501,11 +25753,19 @@
       </c>
       <c r="I347" t="inlineStr">
         <is>
-          <t>- Anthony Thurton and Associates Ltd. BZD $165,093.75 (inclusive of all taxes)</t>
-        </is>
-      </c>
-      <c r="J347" t="inlineStr"/>
-      <c r="K347" t="inlineStr"/>
+          <t>- Anthony Thurton and Associates Ltd. (inclusive of all taxes)</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
+      <c r="K347" t="inlineStr">
+        <is>
+          <t>165093.75</t>
+        </is>
+      </c>
       <c r="L347" t="inlineStr"/>
       <c r="M347" t="inlineStr">
         <is>
@@ -25769,11 +26029,19 @@
       </c>
       <c r="I351" t="inlineStr">
         <is>
-          <t>- Anthony Thurton and Associates Ltd. BZD $182,219.06 (inclusive of taxes)</t>
-        </is>
-      </c>
-      <c r="J351" t="inlineStr"/>
-      <c r="K351" t="inlineStr"/>
+          <t>- Anthony Thurton and Associates Ltd. (inclusive of taxes)</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
+      <c r="K351" t="inlineStr">
+        <is>
+          <t>182219.06</t>
+        </is>
+      </c>
       <c r="L351" t="inlineStr"/>
       <c r="M351" t="inlineStr">
         <is>
@@ -25830,11 +26098,19 @@
       </c>
       <c r="I352" t="inlineStr">
         <is>
-          <t>- CHENTEC BZD $87,004.68 (inclusive of taxes)</t>
-        </is>
-      </c>
-      <c r="J352" t="inlineStr"/>
-      <c r="K352" t="inlineStr"/>
+          <t>- CHENTEC (inclusive of taxes)</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
+      <c r="K352" t="inlineStr">
+        <is>
+          <t>87004.68</t>
+        </is>
+      </c>
       <c r="L352" t="inlineStr"/>
       <c r="M352" t="inlineStr">
         <is>
@@ -25895,12 +26171,24 @@
       </c>
       <c r="I353" t="inlineStr">
         <is>
-          <t>- LF Systems Ltd US$331,900.00, exclusive of local indirect taxes</t>
-        </is>
-      </c>
-      <c r="J353" t="inlineStr"/>
-      <c r="K353" t="inlineStr"/>
-      <c r="L353" t="inlineStr"/>
+          <t>- LF Systems Ltd , exclusive of local indirect taxes</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>US$</t>
+        </is>
+      </c>
+      <c r="K353" t="inlineStr">
+        <is>
+          <t>331900.0</t>
+        </is>
+      </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>331900.0</t>
+        </is>
+      </c>
       <c r="M353" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230303_SLU%20MHWCRP%20Road%20Sector%20Strategy%20Contract%20Award%20Notice%20Rev1.pdf</t>
@@ -27748,7 +28036,7 @@
       <c r="H378" t="inlineStr"/>
       <c r="I378" t="inlineStr">
         <is>
-          <t>CM Construction Supplies- Belize Lot 1: BZ493,031.45 Lot 2:</t>
+          <t>CM Construction Supplies- Belize Lot 1: BZ493,031.45 Lot 2: BZ</t>
         </is>
       </c>
       <c r="J378" t="inlineStr">
@@ -28340,12 +28628,24 @@
       </c>
       <c r="I386" t="inlineStr">
         <is>
-          <t>Formulators Ltd. - Belize BZD 127,466.00 (EURO 57,484.44)</t>
-        </is>
-      </c>
-      <c r="J386" t="inlineStr"/>
-      <c r="K386" t="inlineStr"/>
-      <c r="L386" t="inlineStr"/>
+          <t>Formulators Ltd. - Belize (EURO 57,484.44)</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>BZD</t>
+        </is>
+      </c>
+      <c r="K386" t="inlineStr">
+        <is>
+          <t>127466.0</t>
+        </is>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>63296.99</t>
+        </is>
+      </c>
       <c r="M386" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/Contract%20Award%20Notice.pdf</t>
@@ -29285,16 +29585,24 @@
       <c r="H399" t="inlineStr"/>
       <c r="I399" t="inlineStr">
         <is>
-          <t>Econtec Consultores S.A.S. - Colombia USD $199,</t>
-        </is>
-      </c>
-      <c r="J399" t="inlineStr"/>
+          <t>Econtec Consultores S.A.S. - Colombia</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
       <c r="K399" t="inlineStr">
         <is>
-          <t>240.0</t>
-        </is>
-      </c>
-      <c r="L399" t="inlineStr"/>
+          <t>199240.0</t>
+        </is>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>199240.0</t>
+        </is>
+      </c>
       <c r="M399" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/Contact%20Award%20Information%20Form%20_NURC%20Capacity%20Building%20for%20Tariff%20Review.pdf</t>
@@ -30153,12 +30461,24 @@
       <c r="H411" t="inlineStr"/>
       <c r="I411" t="inlineStr">
         <is>
-          <t>EXP Services Inc. (Canada) in association with C.B. Associates Inc. (Guyana)- Canada and Guyana US$4,029,725.76 (USD 3,381,000 + USD 648,725.76 Indirect Local Taxes)</t>
-        </is>
-      </c>
-      <c r="J411" t="inlineStr"/>
-      <c r="K411" t="inlineStr"/>
-      <c r="L411" t="inlineStr"/>
+          <t>EXP Services Inc. (Canada) in association with C.B. Associates Inc. (Guyana)- Canada and Guyana (USD 3,381,000 + USD 648,725.76 Indirect Local Taxes)</t>
+        </is>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>US$</t>
+        </is>
+      </c>
+      <c r="K411" t="inlineStr">
+        <is>
+          <t>4029725.76</t>
+        </is>
+      </c>
+      <c r="L411" t="inlineStr">
+        <is>
+          <t>4029725.76</t>
+        </is>
+      </c>
       <c r="M411" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/CONTRACT_AWARD_INFORMATION%20%28SERVICE%29_EXP%20.pdf</t>
@@ -30214,7 +30534,7 @@
       <c r="H412" t="inlineStr"/>
       <c r="I412" t="inlineStr">
         <is>
-          <t>Action Construction Equipment (ACE) Private JV. Phoenix Projects Private Ltd. - India Lot 1- GYD 757,673,302 and Lot 2-</t>
+          <t>Action Construction Equipment (ACE) Private JV. Phoenix Projects Private Ltd. - India Lot 1- and Lot 2- GYD 2,130,097,816</t>
         </is>
       </c>
       <c r="J412" t="inlineStr">
@@ -30224,12 +30544,12 @@
       </c>
       <c r="K412" t="inlineStr">
         <is>
-          <t>2130097816.0</t>
+          <t>757673302.0</t>
         </is>
       </c>
       <c r="L412" t="inlineStr">
         <is>
-          <t>10165441.1</t>
+          <t>3615835.51</t>
         </is>
       </c>
       <c r="M412" t="inlineStr">
@@ -30360,12 +30680,24 @@
       <c r="H414" t="inlineStr"/>
       <c r="I414" t="inlineStr">
         <is>
-          <t>Dipcon Engineering Services Ltd. XCD 3,257,900.75 (VAT inclusive)</t>
-        </is>
-      </c>
-      <c r="J414" t="inlineStr"/>
-      <c r="K414" t="inlineStr"/>
-      <c r="L414" t="inlineStr"/>
+          <t>Dipcon Engineering Services Ltd. (VAT inclusive)</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>XCD</t>
+        </is>
+      </c>
+      <c r="K414" t="inlineStr">
+        <is>
+          <t>3257900.75</t>
+        </is>
+      </c>
+      <c r="L414" t="inlineStr">
+        <is>
+          <t>1203440.29</t>
+        </is>
+      </c>
       <c r="M414" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/SJ_SS-PALMISTE%20-%20CONTRACT%20AWARD%20INFORMATION%20%28WORKS%29-02052025.pdf</t>
@@ -30636,12 +30968,24 @@
       <c r="H418" t="inlineStr"/>
       <c r="I418" t="inlineStr">
         <is>
-          <t>CEAC Solutions XCD 351,05.48 (exclusive of taxes)</t>
-        </is>
-      </c>
-      <c r="J418" t="inlineStr"/>
-      <c r="K418" t="inlineStr"/>
-      <c r="L418" t="inlineStr"/>
+          <t>CEAC Solutions ,05.48 (exclusive of taxes)</t>
+        </is>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>XCD</t>
+        </is>
+      </c>
+      <c r="K418" t="inlineStr">
+        <is>
+          <t>351.0</t>
+        </is>
+      </c>
+      <c r="L418" t="inlineStr">
+        <is>
+          <t>129.66</t>
+        </is>
+      </c>
       <c r="M418" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/BSIF%20IV%20Consultancy_CAI.pdf</t>
@@ -30985,12 +31329,24 @@
       <c r="H423" t="inlineStr"/>
       <c r="I423" t="inlineStr">
         <is>
-          <t>H. Lewis Construction Limited XCD 2,097,000 (after a reduction in reduced scope)</t>
-        </is>
-      </c>
-      <c r="J423" t="inlineStr"/>
-      <c r="K423" t="inlineStr"/>
-      <c r="L423" t="inlineStr"/>
+          <t>H. Lewis Construction Limited (after a reduction in reduced scope)</t>
+        </is>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>XCD</t>
+        </is>
+      </c>
+      <c r="K423" t="inlineStr">
+        <is>
+          <t>2097000.0</t>
+        </is>
+      </c>
+      <c r="L423" t="inlineStr">
+        <is>
+          <t>774613.62</t>
+        </is>
+      </c>
       <c r="M423" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/250109%20Contract%20award%20Information%20VSSE.pdf</t>

</xml_diff>

<commit_message>
Apply robust CDB currency parsing and fill BZD/XCD/JA/EUR USD amounts
</commit_message>
<xml_diff>
--- a/data/raw/cdb/cdb_lac_raw.xlsx
+++ b/data/raw/cdb/cdb_lac_raw.xlsx
@@ -1064,7 +1064,11 @@
           <t>1755802.75</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>650297.31</t>
+        </is>
+      </c>
       <c r="M9" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/Contract-Award-Info-ICB-No-20-SFR-OR-STK-01-Nevis-Water-Supply-Pump-Stations.pdf</t>
@@ -2139,7 +2143,11 @@
           <t>1298576.42</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>649288.21</t>
+        </is>
+      </c>
       <c r="M24" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/Contract-Award-Information-Lot-3_George-Price-Highway-Resealing_Belize.pdf</t>
@@ -2208,7 +2216,11 @@
           <t>2539571.76</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>1269785.88</t>
+        </is>
+      </c>
       <c r="M25" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/Contract-Award-Information-Lot-2_George-Price-Highway_-Road-Safety-Furniture-and-Delineation_Belize.pdf</t>
@@ -4800,7 +4812,11 @@
           <t>1176184636.05</t>
         </is>
       </c>
-      <c r="L61" t="inlineStr"/>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>9126800.43</t>
+        </is>
+      </c>
       <c r="M61" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/Fifth-Road-Washington-Boulevard-Project-Jamaica.pdf</t>
@@ -9070,7 +9086,11 @@
           <t>1134920.0</t>
         </is>
       </c>
-      <c r="L119" t="inlineStr"/>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>567460.0</t>
+        </is>
+      </c>
       <c r="M119" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/CONTRACT-AWARD-INFORMATION-Belmopan-Polyclinc.pdf</t>
@@ -9954,7 +9974,11 @@
           <t>1484645.83</t>
         </is>
       </c>
-      <c r="L131" t="inlineStr"/>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>549868.83</t>
+        </is>
+      </c>
       <c r="M131" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/Contract_Award%20Union%20River%20Defense%20issued%20.pdf</t>
@@ -12816,7 +12840,11 @@
           <t>393610.0</t>
         </is>
       </c>
-      <c r="L169" t="inlineStr"/>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>145781.48</t>
+        </is>
+      </c>
       <c r="M169" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/CONTRACT%20AWARD%20INFORMATION_EHRD1_SVG.pdf</t>
@@ -12966,7 +12994,11 @@
           <t>460000.0</t>
         </is>
       </c>
-      <c r="L171" t="inlineStr"/>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>170370.37</t>
+        </is>
+      </c>
       <c r="M171" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/CONTRACT%20AWARD%20INFORMATION_BCAD2_SVG.pdf</t>
@@ -13039,7 +13071,11 @@
           <t>290000.0</t>
         </is>
       </c>
-      <c r="L172" t="inlineStr"/>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>107407.41</t>
+        </is>
+      </c>
       <c r="M172" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/220914_CONTRACT%20AWARD%20INFORMATION_BCAD1_SVG.pdf</t>
@@ -19509,7 +19545,11 @@
           <t>251887.5</t>
         </is>
       </c>
-      <c r="L262" t="inlineStr"/>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>125943.75</t>
+        </is>
+      </c>
       <c r="M262" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/Contract-Award-Information-Consultancy%20Services%20for%20Corazon%20Technical%20High%20School.pdf</t>
@@ -20089,7 +20129,11 @@
           <t>3884905.0</t>
         </is>
       </c>
-      <c r="L270" t="inlineStr"/>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>4082896.02</t>
+        </is>
+      </c>
       <c r="M270" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/220405_SVG_Kingstown%20Port%20Modernisation%20Project_CS_Supervision%20Consultants_2.pdf</t>
@@ -21654,7 +21698,11 @@
           <t>630085.0</t>
         </is>
       </c>
-      <c r="L291" t="inlineStr"/>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>233364.81</t>
+        </is>
+      </c>
       <c r="M291" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230608_GRN_CONTRACT%20AWARD%20INFORMATION%28CONSULTANCY_SERVICES%29%20-%20EHRD_final_0.pdf</t>
@@ -21881,7 +21929,11 @@
           <t>538756.0</t>
         </is>
       </c>
-      <c r="L294" t="inlineStr"/>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>199539.26</t>
+        </is>
+      </c>
       <c r="M294" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230525_CAI%20%28WORKS%29%20St.Vincent%20Grammar%20School%20Lot%203%20.pdf</t>
@@ -22031,7 +22083,11 @@
           <t>136953.0</t>
         </is>
       </c>
-      <c r="L296" t="inlineStr"/>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>68476.5</t>
+        </is>
+      </c>
       <c r="M296" t="inlineStr"/>
       <c r="N296" t="inlineStr">
         <is>
@@ -22177,7 +22233,11 @@
           <t>3008779.92</t>
         </is>
       </c>
-      <c r="L298" t="inlineStr"/>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>1114362.93</t>
+        </is>
+      </c>
       <c r="M298" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230427_SLU_EQuIP_SALCC%20Renovation.pdf</t>
@@ -22319,7 +22379,11 @@
           <t>242720.33</t>
         </is>
       </c>
-      <c r="L300" t="inlineStr"/>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>121360.16</t>
+        </is>
+      </c>
       <c r="M300" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230424_BZE_CAI%20Consultancy%20Services%20for%20Cristo%20Rey%20RC%20Pre-Primary%20and%20Primary%20School_Variation.pdf</t>
@@ -22388,7 +22452,11 @@
           <t>370644.42</t>
         </is>
       </c>
-      <c r="L301" t="inlineStr"/>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>185322.21</t>
+        </is>
+      </c>
       <c r="M301" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230424_BZE_CAI_Consultancy%20Services%20for%20Corazon%20Technical%20High%20School.pdf</t>
@@ -23126,7 +23194,11 @@
           <t>6060539.03</t>
         </is>
       </c>
-      <c r="L311" t="inlineStr"/>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>2244644.09</t>
+        </is>
+      </c>
       <c r="M311" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230330_SVG_CAI%20%28WORKS%29%20-Mesopotamia%20Community%20Centre%20.pdf</t>
@@ -23195,7 +23267,11 @@
           <t>3539883.14</t>
         </is>
       </c>
-      <c r="L312" t="inlineStr"/>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>1311067.83</t>
+        </is>
+      </c>
       <c r="M312" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230330_SVG_CAI%20%28WORKS%29%20-%20Yambou%20and%20Teviot%20River%20Defense%20and%20Training%20Works%20Mesopotamia%20_0.pdf</t>
@@ -23264,7 +23340,11 @@
           <t>2069326.0</t>
         </is>
       </c>
-      <c r="L313" t="inlineStr"/>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>766417.04</t>
+        </is>
+      </c>
       <c r="M313" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230330_SVG_WORKS%20-%20Union%20River%20Defense%20Training%20Works%20.pdf</t>
@@ -24298,7 +24378,11 @@
           <t>351123.76</t>
         </is>
       </c>
-      <c r="L327" t="inlineStr"/>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>175561.88</t>
+        </is>
+      </c>
       <c r="M327" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230327_BZE_CAI%20-%20Dorothy%20Menzies%20Child%20Care%20Center%20Replacement%20%28Consultancy%29.pdf</t>
@@ -24517,7 +24601,11 @@
           <t>30000.0</t>
         </is>
       </c>
-      <c r="L330" t="inlineStr"/>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>15000.0</t>
+        </is>
+      </c>
       <c r="M330" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230323_BZE_CONTRACT%20AWARD%20INFO_CONSULTANCY_SERVICES-%20Belize%20Red%20Cross-%20KAP.pdf</t>
@@ -24809,7 +24897,11 @@
           <t>454800.0</t>
         </is>
       </c>
-      <c r="L334" t="inlineStr"/>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>168444.44</t>
+        </is>
+      </c>
       <c r="M334" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230314_SVG_CONTRACT%20AWARD%20INFORMATION%28CONSULTANCY_SERVICES%29-%20Perseverance%20Road.pdf</t>
@@ -24951,7 +25043,11 @@
           <t>368334.8</t>
         </is>
       </c>
-      <c r="L336" t="inlineStr"/>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>184167.4</t>
+        </is>
+      </c>
       <c r="M336" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230313_BZE_Consultancy_Second%20Road%20Safety%20Project.pdf</t>
@@ -25020,7 +25116,11 @@
           <t>29555.99</t>
         </is>
       </c>
-      <c r="L337" t="inlineStr"/>
+      <c r="L337" t="inlineStr">
+        <is>
+          <t>14778.0</t>
+        </is>
+      </c>
       <c r="M337" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230315_BZE_CAI_Goods-%20FOR%20SUPPY%20AND%20DELIVERY%20ITNEQUIPMENT%20FOR%20MARIA%20CRAWFORD%20HEALTH%20CENTER%20-CROOKED%20TREE%20VILLAGE%20-BELIZE%20DISTRICT.pdf</t>
@@ -25628,7 +25728,11 @@
           <t>154849.5</t>
         </is>
       </c>
-      <c r="L345" t="inlineStr"/>
+      <c r="L345" t="inlineStr">
+        <is>
+          <t>77424.75</t>
+        </is>
+      </c>
       <c r="M345" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230315_CAI_CONSULTANCY_SERVICES-%20YEC%20Santa%20Cruz%20BNTF10.pdf</t>
@@ -25697,7 +25801,11 @@
           <t>189787.5</t>
         </is>
       </c>
-      <c r="L346" t="inlineStr"/>
+      <c r="L346" t="inlineStr">
+        <is>
+          <t>94893.75</t>
+        </is>
+      </c>
       <c r="M346" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230315_BZE_CAI_CONSULTANCY_SERVICES-%20ATA%20Mabil%20Ha%20%20BNTF10%20%28002%29.pdf</t>
@@ -25766,7 +25874,11 @@
           <t>165093.75</t>
         </is>
       </c>
-      <c r="L347" t="inlineStr"/>
+      <c r="L347" t="inlineStr">
+        <is>
+          <t>82546.88</t>
+        </is>
+      </c>
       <c r="M347" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230315_BZE_CAI_CONSULTANCY_SERVICES-%20ATA%20Mafredi%20BNTF10.pdf</t>
@@ -26042,7 +26154,11 @@
           <t>182219.06</t>
         </is>
       </c>
-      <c r="L351" t="inlineStr"/>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>91109.53</t>
+        </is>
+      </c>
       <c r="M351" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230313_BZE_CAI_CONSULTANCY_SERVICES-%20ATA%20Gales%20Point%20-%20BNTF10.pdf</t>
@@ -26111,7 +26227,11 @@
           <t>87004.68</t>
         </is>
       </c>
-      <c r="L352" t="inlineStr"/>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>43502.34</t>
+        </is>
+      </c>
       <c r="M352" t="inlineStr">
         <is>
           <t>https://www.caribank.org/sites/default/files/publication-resources/230313_Belize%20Social%20Investment%20Fund%20III_CAI_CONSULTANCY_SERVICES-%20CHENTEC%20.pdf</t>
@@ -27617,7 +27737,7 @@
       </c>
       <c r="L372" t="inlineStr">
         <is>
-          <t>270622.23</t>
+          <t>281369.02</t>
         </is>
       </c>
       <c r="M372" t="inlineStr">
@@ -27690,7 +27810,7 @@
       </c>
       <c r="L373" t="inlineStr">
         <is>
-          <t>640857.57</t>
+          <t>645272.0</t>
         </is>
       </c>
       <c r="M373" t="inlineStr">
@@ -27836,7 +27956,7 @@
       </c>
       <c r="L375" t="inlineStr">
         <is>
-          <t>516470.57</t>
+          <t>517369.93</t>
         </is>
       </c>
       <c r="M375" t="inlineStr">
@@ -27909,7 +28029,7 @@
       </c>
       <c r="L376" t="inlineStr">
         <is>
-          <t>526856.33</t>
+          <t>527773.77</t>
         </is>
       </c>
       <c r="M376" t="inlineStr">
@@ -27978,7 +28098,7 @@
       </c>
       <c r="L377" t="inlineStr">
         <is>
-          <t>103356.87</t>
+          <t>107461.32</t>
         </is>
       </c>
       <c r="M377" t="inlineStr">
@@ -28124,7 +28244,7 @@
       </c>
       <c r="L379" t="inlineStr">
         <is>
-          <t>36686.49</t>
+          <t>38143.36</t>
         </is>
       </c>
       <c r="M379" t="inlineStr">
@@ -28197,7 +28317,7 @@
       </c>
       <c r="L380" t="inlineStr">
         <is>
-          <t>59859.55</t>
+          <t>62236.66</t>
         </is>
       </c>
       <c r="M380" t="inlineStr">
@@ -28420,7 +28540,7 @@
       </c>
       <c r="L383" t="inlineStr">
         <is>
-          <t>59832.95</t>
+          <t>62209.0</t>
         </is>
       </c>
       <c r="M383" t="inlineStr">
@@ -28643,7 +28763,7 @@
       </c>
       <c r="L386" t="inlineStr">
         <is>
-          <t>63296.99</t>
+          <t>63733.0</t>
         </is>
       </c>
       <c r="M386" t="inlineStr">
@@ -28789,7 +28909,7 @@
       </c>
       <c r="L388" t="inlineStr">
         <is>
-          <t>14279.96</t>
+          <t>14378.33</t>
         </is>
       </c>
       <c r="M388" t="inlineStr">
@@ -28935,7 +29055,7 @@
       </c>
       <c r="L390" t="inlineStr">
         <is>
-          <t>494772.39</t>
+          <t>475083.99</t>
         </is>
       </c>
       <c r="M390" t="inlineStr">
@@ -29012,7 +29132,7 @@
       </c>
       <c r="L391" t="inlineStr">
         <is>
-          <t>682897.75</t>
+          <t>689953.98</t>
         </is>
       </c>
       <c r="M391" t="inlineStr">
@@ -29085,7 +29205,7 @@
       </c>
       <c r="L392" t="inlineStr">
         <is>
-          <t>189032.64</t>
+          <t>181510.49</t>
         </is>
       </c>
       <c r="M392" t="inlineStr">
@@ -29673,7 +29793,7 @@
       </c>
       <c r="L400" t="inlineStr">
         <is>
-          <t>22308.2</t>
+          <t>21420.49</t>
         </is>
       </c>
       <c r="M400" t="inlineStr">
@@ -29819,7 +29939,7 @@
       </c>
       <c r="L402" t="inlineStr">
         <is>
-          <t>266721.02</t>
+          <t>256107.43</t>
         </is>
       </c>
       <c r="M402" t="inlineStr">
@@ -29892,7 +30012,7 @@
       </c>
       <c r="L403" t="inlineStr">
         <is>
-          <t>108095.64</t>
+          <t>105752.72</t>
         </is>
       </c>
       <c r="M403" t="inlineStr">
@@ -29965,7 +30085,7 @@
       </c>
       <c r="L404" t="inlineStr">
         <is>
-          <t>73828.4</t>
+          <t>70890.56</t>
         </is>
       </c>
       <c r="M404" t="inlineStr">
@@ -30184,7 +30304,7 @@
       </c>
       <c r="L407" t="inlineStr">
         <is>
-          <t>172968.74</t>
+          <t>166085.82</t>
         </is>
       </c>
       <c r="M407" t="inlineStr">
@@ -30622,7 +30742,7 @@
       </c>
       <c r="L413" t="inlineStr">
         <is>
-          <t>43148335.31</t>
+          <t>43262696.31</t>
         </is>
       </c>
       <c r="M413" t="inlineStr">
@@ -30695,7 +30815,7 @@
       </c>
       <c r="L414" t="inlineStr">
         <is>
-          <t>1203440.29</t>
+          <t>1206629.91</t>
         </is>
       </c>
       <c r="M414" t="inlineStr">
@@ -30768,7 +30888,7 @@
       </c>
       <c r="L415" t="inlineStr">
         <is>
-          <t>849763.69</t>
+          <t>852015.92</t>
         </is>
       </c>
       <c r="M415" t="inlineStr">
@@ -30841,7 +30961,7 @@
       </c>
       <c r="L416" t="inlineStr">
         <is>
-          <t>1078276.84</t>
+          <t>1081134.72</t>
         </is>
       </c>
       <c r="M416" t="inlineStr">
@@ -30914,7 +31034,7 @@
       </c>
       <c r="L417" t="inlineStr">
         <is>
-          <t>3692052.05</t>
+          <t>3701837.52</t>
         </is>
       </c>
       <c r="M417" t="inlineStr">
@@ -30983,7 +31103,7 @@
       </c>
       <c r="L418" t="inlineStr">
         <is>
-          <t>129.66</t>
+          <t>130.0</t>
         </is>
       </c>
       <c r="M418" t="inlineStr">
@@ -31129,7 +31249,7 @@
       </c>
       <c r="L420" t="inlineStr">
         <is>
-          <t>1799408.77</t>
+          <t>1727805.16</t>
         </is>
       </c>
       <c r="M420" t="inlineStr">
@@ -31202,7 +31322,7 @@
       </c>
       <c r="L421" t="inlineStr">
         <is>
-          <t>72003.36</t>
+          <t>72194.2</t>
         </is>
       </c>
       <c r="M421" t="inlineStr">
@@ -31344,7 +31464,7 @@
       </c>
       <c r="L423" t="inlineStr">
         <is>
-          <t>774613.62</t>
+          <t>776666.67</t>
         </is>
       </c>
       <c r="M423" t="inlineStr">
@@ -31413,7 +31533,7 @@
       </c>
       <c r="L424" t="inlineStr">
         <is>
-          <t>530431.01</t>
+          <t>531836.87</t>
         </is>
       </c>
       <c r="M424" t="inlineStr">
@@ -31482,7 +31602,7 @@
       </c>
       <c r="L425" t="inlineStr">
         <is>
-          <t>863386.43</t>
+          <t>865674.76</t>
         </is>
       </c>
       <c r="M425" t="inlineStr">
@@ -31555,7 +31675,7 @@
       </c>
       <c r="L426" t="inlineStr">
         <is>
-          <t>142065.21</t>
+          <t>142441.74</t>
         </is>
       </c>
       <c r="M426" t="inlineStr">
@@ -31628,7 +31748,7 @@
       </c>
       <c r="L427" t="inlineStr">
         <is>
-          <t>483888.59</t>
+          <t>488888.5</t>
         </is>
       </c>
       <c r="M427" t="inlineStr">
@@ -31701,7 +31821,7 @@
       </c>
       <c r="L428" t="inlineStr">
         <is>
-          <t>584184.34</t>
+          <t>590220.58</t>
         </is>
       </c>
       <c r="M428" t="inlineStr">

</xml_diff>